<commit_message>
Rebuild group 1 (Power) from the wire lists: CabinPower, EngineRoom-C, HeavyDC, RearFuel
build_harness.py keeps line endings, copies missing wire parts from the library, no empty cables.
Wiring diagrams read fuse name / rating from the fuse box spec, not the cavity text.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/AntiTheft-wirelist.xlsx
+++ b/docs/harness/wirelist/AntiTheft-wirelist.xlsx
@@ -2386,7 +2386,7 @@
       </c>
       <c r="R14" s="47" t="inlineStr">
         <is>
-          <t>+12V ALMS 2A (LOGIC BUS1-8)</t>
+          <t>+12V Shock sensor +12 V (LOGIC BUS1-8)</t>
         </is>
       </c>
       <c r="S14" s="48" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="R15" s="31" t="inlineStr">
         <is>
-          <t>+12V ALM 5A (LOGIC BUS1-7)</t>
+          <t>+12V Alarm +12 V (LOGIC BUS1-7)</t>
         </is>
       </c>
       <c r="S15" s="32" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="R18" s="47" t="inlineStr">
         <is>
-          <t>+12V ALMIG 2A (LOGIC BUS2-9)</t>
+          <t>+12V Alarm ignition +12V (LOGIC BUS2-9)</t>
         </is>
       </c>
       <c r="S18" s="48" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="E3" s="31" t="inlineStr">
         <is>
-          <t>+12V ALM 5A (LOGIC BUS1-7)</t>
+          <t>+12V Alarm +12 V (LOGIC BUS1-7)</t>
         </is>
       </c>
       <c r="F3" s="32" t="n">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="E4" s="47" t="inlineStr">
         <is>
-          <t>+12V ALMIG 2A (LOGIC BUS2-9)</t>
+          <t>+12V Alarm ignition +12V (LOGIC BUS2-9)</t>
         </is>
       </c>
       <c r="F4" s="48" t="n">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="E9" s="31" t="inlineStr">
         <is>
-          <t>+12V ALMS 2A (LOGIC BUS1-8)</t>
+          <t>+12V Shock sensor +12 V (LOGIC BUS1-8)</t>
         </is>
       </c>
       <c r="F9" s="32" t="n">

</xml_diff>

<commit_message>
Rebuild group 1 (Power) from the wire lists: CabinPower, EngineRoom-C, HeavyDC, RearFuel (#342)
build_harness.py keeps line endings, copies missing wire parts from the library, no empty cables.
Wiring diagrams read fuse name / rating from the fuse box spec, not the cavity text.

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/AntiTheft-wirelist.xlsx
+++ b/docs/harness/wirelist/AntiTheft-wirelist.xlsx
@@ -2386,7 +2386,7 @@
       </c>
       <c r="R14" s="47" t="inlineStr">
         <is>
-          <t>+12V ALMS 2A (LOGIC BUS1-8)</t>
+          <t>+12V Shock sensor +12 V (LOGIC BUS1-8)</t>
         </is>
       </c>
       <c r="S14" s="48" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="R15" s="31" t="inlineStr">
         <is>
-          <t>+12V ALM 5A (LOGIC BUS1-7)</t>
+          <t>+12V Alarm +12 V (LOGIC BUS1-7)</t>
         </is>
       </c>
       <c r="S15" s="32" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="R18" s="47" t="inlineStr">
         <is>
-          <t>+12V ALMIG 2A (LOGIC BUS2-9)</t>
+          <t>+12V Alarm ignition +12V (LOGIC BUS2-9)</t>
         </is>
       </c>
       <c r="S18" s="48" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="E3" s="31" t="inlineStr">
         <is>
-          <t>+12V ALM 5A (LOGIC BUS1-7)</t>
+          <t>+12V Alarm +12 V (LOGIC BUS1-7)</t>
         </is>
       </c>
       <c r="F3" s="32" t="n">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="E4" s="47" t="inlineStr">
         <is>
-          <t>+12V ALMIG 2A (LOGIC BUS2-9)</t>
+          <t>+12V Alarm ignition +12V (LOGIC BUS2-9)</t>
         </is>
       </c>
       <c r="F4" s="48" t="n">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="E9" s="31" t="inlineStr">
         <is>
-          <t>+12V ALMS 2A (LOGIC BUS1-8)</t>
+          <t>+12V Shock sensor +12 V (LOGIC BUS1-8)</t>
         </is>
       </c>
       <c r="F9" s="32" t="n">

</xml_diff>

<commit_message>
WIP: merge loom A + B into ECU-cabin / ECU-engine (drawings, lists, registry, gates)
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/AntiTheft-wirelist.xlsx
+++ b/docs/harness/wirelist/AntiTheft-wirelist.xlsx
@@ -1664,7 +1664,7 @@
       </c>
       <c r="D8" s="39" t="inlineStr">
         <is>
-          <t>B-cabin</t>
+          <t>ECU-cabin</t>
         </is>
       </c>
       <c r="E8" s="40" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="AG8" s="54" t="inlineStr">
         <is>
-          <t>owner proposed: longer half (drawn today as w_at_immob2_bc on B-cabin, 120 mm; w_at_immob2 on AntiTheft, 1210 mm)</t>
+          <t>owner proposed: longer half (drawn today as w_at_immob2_bc on ECU-cabin, 120 mm; w_at_immob2 on AntiTheft, 1210 mm)</t>
         </is>
       </c>
     </row>

</xml_diff>